<commit_message>
Rapport des tests d'écran : état de 9 h 50 (364 / 422)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
+++ b/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -557,7 +557,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>422 tests : 358 OK, 64 en échec</t>
+          <t>422 tests : 364 OK, 58 en échec</t>
         </is>
       </c>
     </row>
@@ -641,10 +641,10 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1041,10 +1041,10 @@
         <v>282</v>
       </c>
       <c r="C33" t="n">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="D33" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34">
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="41">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
@@ -1173,16 +1173,6 @@
       </c>
       <c r="B44" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Défaut ouvert</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4308,7 +4298,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>282 tests, 238 OK, 44 en échec</t>
+          <t>282 tests, 243 OK, 39 en échec</t>
         </is>
       </c>
     </row>
@@ -4974,27 +4964,19 @@
           <t>retours/test-connexion-bouton-pointage.js</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>10 / 10</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -9458,27 +9440,19 @@
           <t>retours/test-rh-badge-carte-par-page.js</t>
         </is>
       </c>
-      <c r="B241" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C241" s="5" t="inlineStr"/>
-      <c r="D241" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E241" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F241" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+      <c r="B241" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C241" s="5" t="inlineStr">
+        <is>
+          <t>6 / 6</t>
+        </is>
+      </c>
+      <c r="D241" s="5" t="inlineStr"/>
+      <c r="E241" s="5" t="inlineStr"/>
+      <c r="F241" s="5" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="5" t="inlineStr">
@@ -9486,27 +9460,19 @@
           <t>retours/test-rh-badge-qr.js</t>
         </is>
       </c>
-      <c r="B242" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C242" s="5" t="inlineStr"/>
-      <c r="D242" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E242" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F242" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+      <c r="B242" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C242" s="5" t="inlineStr">
+        <is>
+          <t>15 / 15</t>
+        </is>
+      </c>
+      <c r="D242" s="5" t="inlineStr"/>
+      <c r="E242" s="5" t="inlineStr"/>
+      <c r="F242" s="5" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="5" t="inlineStr">
@@ -9519,7 +9485,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="C243" s="5" t="inlineStr"/>
+      <c r="C243" s="5" t="inlineStr">
+        <is>
+          <t>14 / 14</t>
+        </is>
+      </c>
       <c r="D243" s="5" t="inlineStr"/>
       <c r="E243" s="5" t="inlineStr"/>
       <c r="F243" s="5" t="inlineStr"/>
@@ -9570,31 +9540,19 @@
           <t>retours/test-rh.js</t>
         </is>
       </c>
-      <c r="B246" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B246" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C246" s="5" t="inlineStr">
         <is>
-          <t>48 / 49</t>
-        </is>
-      </c>
-      <c r="D246" s="5" t="inlineStr">
-        <is>
-          <t>Utilisateurs actifs créés et rattachés comme employés à l'ouverture (hors admin)  [1]</t>
-        </is>
-      </c>
-      <c r="E246" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F246" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+          <t>49 / 49</t>
+        </is>
+      </c>
+      <c r="D246" s="5" t="inlineStr"/>
+      <c r="E246" s="5" t="inlineStr"/>
+      <c r="F246" s="5" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="5" t="inlineStr">
@@ -10362,27 +10320,19 @@
           <t>retours/test-whatsapp-session-alerte.js</t>
         </is>
       </c>
-      <c r="B282" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C282" s="5" t="inlineStr"/>
-      <c r="D282" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E282" s="5" t="inlineStr">
-        <is>
-          <t>Configuration du poste</t>
-        </is>
-      </c>
-      <c r="F282" s="5" t="inlineStr">
-        <is>
-          <t>Service WhatsApp Web non installé sur le poste.</t>
-        </is>
-      </c>
+      <c r="B282" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="inlineStr">
+        <is>
+          <t>12 / 12</t>
+        </is>
+      </c>
+      <c r="D282" s="5" t="inlineStr"/>
+      <c r="E282" s="5" t="inlineStr"/>
+      <c r="F282" s="5" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="5" t="inlineStr">
@@ -11638,7 +11588,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14 tests, 13 OK, 1 en échec</t>
+          <t>14 tests, 14 OK, 0 en échec</t>
         </is>
       </c>
     </row>
@@ -11780,31 +11730,19 @@
           <t>audits/repro-vente-assurance.js</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>16 / 17</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>CR-04 attendu : 3 paires de clôtures simultanées sur le même organisme → encours = somme des parts  [clôtures réussies 6/6 ; somme des parts 3384 ; encours organisme 1692 ; encours client 1692]</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Défaut ouvert</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>CR-04 : deux clôtures simultanées sur le même organisme écrasent l'encours (lecture puis écriture en Java). Correction proposée : addition faite par la base, en une requête.</t>
-        </is>
-      </c>
+          <t>17 / 17</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -11937,11 +11875,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>10 / 10</t>
-        </is>
-      </c>
+      <c r="C16" s="5" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Rapport des tests d'écran : série complète du 30/10 (352 / 422)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
+++ b/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
@@ -557,7 +557,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>422 tests : 364 OK, 58 en échec</t>
+          <t>422 tests : 352 OK, 70 en échec</t>
         </is>
       </c>
     </row>
@@ -625,10 +625,10 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -641,10 +641,10 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -673,10 +673,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -865,10 +865,10 @@
         <v>12</v>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -977,10 +977,10 @@
         <v>6</v>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1041,10 +1041,10 @@
         <v>282</v>
       </c>
       <c r="C33" t="n">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D33" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34">
@@ -1057,10 +1057,10 @@
         <v>13</v>
       </c>
       <c r="C34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1132,37 +1132,37 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Configuration du poste</t>
+          <t>Données de la copie</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Données de la copie</t>
+          <t>Lenteur (grosse base)</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lenteur (grosse base)</t>
+          <t>Configuration du poste</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -2149,7 +2149,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12 tests, 11 OK, 1 en échec</t>
+          <t>12 tests, 9 OK, 3 en échec</t>
         </is>
       </c>
     </row>
@@ -2211,17 +2211,21 @@
           <t>journal/test-export-journal.js</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>10 / 10</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr"/>
+          <t>3 / 6</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>le bouton declenche bien un telechargement  [aucun]</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
@@ -2291,17 +2295,21 @@
           <t>journal/test-scan-qr-publicitaire.js</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>13 / 13</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr"/>
+          <t>11 / 13</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Vente dépôt : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé  [{"champ":"htt","fenetre":false,"texte":false} appels : ]</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
     </row>
@@ -2879,7 +2887,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>v1/checkproduit (tout) : réponse en moins de 20 s  [50990 ms, 11650]</t>
+          <t>v1/checkproduit (tout) : réponse en moins de 20 s  [58625 ms, 11650]</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -3003,12 +3011,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>2 / 3</t>
+          <t>1 / 3</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Réponse 200 en moins de 30 s, un produit par article (193 articles détail sans indicateur)  [200, 120670 ms, 22112 / 22112]</t>
+          <t>Réponse 200 en moins de 30 s, un produit par article (193 articles détail sans indicateur)  [200, 133642 ms, 22112 / 22112]</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -3557,7 +3565,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6 tests, 6 OK, 0 en échec</t>
+          <t>6 tests, 4 OK, 2 en échec</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3607,21 @@
           <t>productivite/test-activite-equipes-analyses.js</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>11 / 11</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
+          <t>10 / 11</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Parcours sans exception  [page.fill: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
@@ -3619,17 +3631,21 @@
           <t>productivite/test-activite-equipes-donnees.js</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>11 / 11</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr"/>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Parcours sans exception  [locator.click: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
@@ -4298,7 +4314,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>282 tests, 243 OK, 39 en échec</t>
+          <t>282 tests, 233 OK, 49 en échec</t>
         </is>
       </c>
     </row>
@@ -4836,17 +4852,21 @@
           <t>retours/test-commande-en-cours-0825.js</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>5 / 5</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
+          <t>1 / 2</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Parcours sans exception  [locator.click: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
       <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="5" t="inlineStr"/>
     </row>
@@ -4924,17 +4944,21 @@
           <t>retours/test-connexion-badge-lecture.js</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>11 / 11</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr"/>
+          <t>8 / 10</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>QWERTY et verrouillage majuscules (« PRESTIGE°BQDGE*1*WWL°2… ») : connexion par le bouton badge  [http://localhost:8080/prestige/security/index.html]</t>
+        </is>
+      </c>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
     </row>
@@ -5328,17 +5352,21 @@
           <t>retours/test-differes-modification.js</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>13 / 13</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr"/>
+          <t>12 / 12</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>arrêt du test (code 1) sans contrôle en échec</t>
+        </is>
+      </c>
       <c r="E49" s="5" t="inlineStr"/>
       <c r="F49" s="5" t="inlineStr"/>
     </row>
@@ -5628,17 +5656,21 @@
           <t>retours/test-etiquettes-gs1.js</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>17 / 17</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr"/>
+          <t>1 / 3</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
+        </is>
+      </c>
       <c r="E64" s="5" t="inlineStr"/>
       <c r="F64" s="5" t="inlineStr"/>
     </row>
@@ -5648,17 +5680,21 @@
           <t>retours/test-etiquettes-personnalisation.js</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>50 / 50</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr"/>
+          <t>1 / 2</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
+        </is>
+      </c>
       <c r="E65" s="5" t="inlineStr"/>
       <c r="F65" s="5" t="inlineStr"/>
     </row>
@@ -5912,17 +5948,21 @@
           <t>retours/test-fidelite-vente-utiliser.js</t>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>12 / 12</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr"/>
+          <t>11 / 11</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>arrêt du test (code 1) sans contrôle en échec</t>
+        </is>
+      </c>
       <c r="E77" s="5" t="inlineStr"/>
       <c r="F77" s="5" t="inlineStr"/>
     </row>
@@ -6020,17 +6060,21 @@
           <t>retours/test-gs1-bascule.js</t>
         </is>
       </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>25 / 25</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr"/>
+          <t>2 / 4</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
+        </is>
+      </c>
       <c r="E82" s="5" t="inlineStr"/>
       <c r="F82" s="5" t="inlineStr"/>
     </row>
@@ -6040,17 +6084,21 @@
           <t>retours/test-gs1-controle-lot.js</t>
         </is>
       </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>25 / 25</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr"/>
+          <t>2 / 4</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
+        </is>
+      </c>
       <c r="E83" s="5" t="inlineStr"/>
       <c r="F83" s="5" t="inlineStr"/>
     </row>
@@ -6424,17 +6472,21 @@
           <t>retours/test-journal-complet.js</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>18 / 18</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr"/>
+          <t>1 / 3</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
+        </is>
+      </c>
       <c r="E101" s="5" t="inlineStr"/>
       <c r="F101" s="5" t="inlineStr"/>
     </row>
@@ -6551,12 +6603,12 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>2 / 3</t>
+          <t>13 / 15</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Déroulement du test  [page.evaluate: Target crashed</t>
+          <t>(g) 10 erreurs identiques simultanées : un seul événement, 10 occurrences (aucune perdue)  [0|0]</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -6748,17 +6800,21 @@
           <t>retours/test-lot-l.js</t>
         </is>
       </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>31 / 31</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr"/>
+          <t>30 / 31</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>jeu d essai pose sur une fenetre vierge (2023-10-01 .. 2023-11-30)  [mouvements preexistants=10]</t>
+        </is>
+      </c>
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="5" t="inlineStr"/>
     </row>
@@ -6773,7 +6829,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr"/>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>24 / 24</t>
+        </is>
+      </c>
       <c r="D117" s="5" t="inlineStr"/>
       <c r="E117" s="5" t="inlineStr"/>
       <c r="F117" s="5" t="inlineStr"/>
@@ -7268,7 +7328,7 @@
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>Avec le jeton : profil, droit photos, pas de pointage sans employé  [{"utilisateur":{"id":"90000000000000000001","login":"e2e","nom":"Essai E2E"},"employe":{"matricule":"e2e","id":"d3fe3b44-2f0a-4aaa-a272-ef7465d4a322","nom":"Essai E2E"},"success":true,"pointage":{"qr":true,"gps":false},"droits":{"pointage":true,"photos":true}}]</t>
+          <t>Avec le jeton : profil, droit photos, pas de pointage sans employé  [{"utilisateur":{"id":"90000000000000000001","login":"e2e","nom":"Essai E2E"},"employe":{"matricule":"E2E-BL-M1","id":"E2E-BL-1","nom":"ESSAI Badge lecture"},"success":true,"pointage":{"qr":true,"gps":false},"droits":{"pointage":true,"photos":true}}]</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
@@ -7524,7 +7584,7 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>Elle porte la traçabilité : la saisie, sa date et son auteur  [s) (SIROP NON TENU) (1) () (5 ml le soir) (10 jours) (POMMADE PRESCRITE) (3) () (application locale) (15 jours) (TOTAL : 3 produit\(s\) prescrit\(s\)) (OBSERVATIONS) (Contrôle dans trois mois. Surveiller la tension.) (Saisie le 30/10/2026 07:43 par Essai E2E) (RC N° CI-TDI-2022-B-1010 - CC N° 2245364C - Centre des Impôts: YAMO]</t>
+          <t>Elle porte la traçabilité : la saisie, sa date et son auteur  [s) (SIROP NON TENU) (1) () (5 ml le soir) (10 jours) (POMMADE PRESCRITE) (3) () (application locale) (15 jours) (TOTAL : 3 produit\(s\) prescrit\(s\)) (OBSERVATIONS) (Contrôle dans trois mois. Surveiller la tension.) (Saisie le 30/10/2026 12:38 par Essai E2E) (RC N° CI-TDI-2022-B-1010 - CC N° 2245364C - Centre des Impôts: YAMO]</t>
         </is>
       </c>
       <c r="E152" s="5" t="inlineStr">
@@ -7716,7 +7776,7 @@
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>Le parcours va au bout  [Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-30283.cnf --default-character-set=utf8mb4 laborex_v1_db -e INSERT INTO t_famille_dci (lg_FAMILLE_DCI_ID, lg_FAMILLE_ID, lg_DCI_ID, str_STATUT, dt_CREATED, dt_UPDATED) SELECT CONCAT('E2E-SUB-', 0), f.lg_FAMILLE_ID,</t>
+          <t xml:space="preserve">Le parcours va au bout  [Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -e INSERT INTO t_famille_dci (lg_FAMILLE_DCI_ID, lg_FAMILLE_ID, lg_DCI_ID, str_STATUT, dt_CREATED, dt_UPDATED) SELECT CONCAT('E2E-SUB-', 0), f.lg_FAMILLE_ID, </t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
@@ -7756,17 +7816,17 @@
           <t>retours/test-paiement-points.js</t>
         </is>
       </c>
-      <c r="B163" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="C163" s="5" t="inlineStr">
-        <is>
-          <t>25 / 25</t>
-        </is>
-      </c>
-      <c r="D163" s="5" t="inlineStr"/>
+      <c r="B163" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr"/>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>arrêt du test (code 1) sans contrôle en échec</t>
+        </is>
+      </c>
       <c r="E163" s="5" t="inlineStr"/>
       <c r="F163" s="5" t="inlineStr"/>
     </row>
@@ -8012,7 +8072,7 @@
       </c>
       <c r="D174" s="5" t="inlineStr">
         <is>
-          <t>Envoi (écran) : « a bien reçu la commande », pas d'échec ; en-tête de contrôle correct  [Envoi PharmaMLDPCI a bien reçu la commande. Sa réponse (quantités livrées, ruptures) n'est pas immédiate : elle sera récupérée automatiquement, ou par le bouton « Réponses PharmaML ». Ne renvoyez pas la commande.  OKOuiNonAnnuler[{"nature":"REQ_EMISSION","action":"COMMANDE","ref":"20261030074514","enRep":"","c</t>
+          <t>Envoi (écran) : « a bien reçu la commande », pas d'échec ; en-tête de contrôle correct  [Envoi PharmaMLDPCI a bien reçu la commande. Sa réponse (quantités livrées, ruptures) n'est pas immédiate : elle sera récupérée automatiquement, ou par le bouton « Réponses PharmaML ». Ne renvoyez pas la commande.  OKOuiNonAnnuler[{"nature":"REQ_EMISSION","action":"COMMANDE","ref":"20261030124508","enRep":"","c</t>
         </is>
       </c>
       <c r="E174" s="5" t="inlineStr">
@@ -8576,7 +8636,7 @@
       </c>
       <c r="D201" s="5" t="inlineStr">
         <is>
-          <t>Le parcours va au bout  [Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-30283.cnf --default-character-set=utf8mb4 laborex_v1_db -e INSERT INTO t_famille_dci (lg_FAMILLE_DCI_ID, lg_FAMILLE_ID, lg_DCI_ID, str_STATUT, dt_CREATED, dt_UPDATED) SELECT 'E2E-EQV-0', f.lg_FAMILLE_ID, '', 'enab</t>
+          <t>Le parcours va au bout  [Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -e INSERT INTO t_famille_dci (lg_FAMILLE_DCI_ID, lg_FAMILLE_ID, lg_DCI_ID, str_STATUT, dt_CREATED, dt_UPDATED) SELECT 'E2E-EQV-0', f.lg_FAMILLE_ID, '', 'enabl</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
@@ -8708,31 +8768,19 @@
           <t>retours/test-prevente.js</t>
         </is>
       </c>
-      <c r="B207" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B207" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C207" s="5" t="inlineStr">
         <is>
-          <t>9 / 9</t>
-        </is>
-      </c>
-      <c r="D207" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 124) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E207" s="5" t="inlineStr">
-        <is>
-          <t>Lenteur (grosse base)</t>
-        </is>
-      </c>
-      <c r="F207" s="5" t="inlineStr">
-        <is>
-          <t>Dépasse 15 minutes sur la grosse base.</t>
-        </is>
-      </c>
+          <t>16 / 16</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr"/>
+      <c r="E207" s="5" t="inlineStr"/>
+      <c r="F207" s="5" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="5" t="inlineStr">
@@ -8937,7 +8985,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="C217" s="5" t="inlineStr"/>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>15 / 15</t>
+        </is>
+      </c>
       <c r="D217" s="5" t="inlineStr"/>
       <c r="E217" s="5" t="inlineStr"/>
       <c r="F217" s="5" t="inlineStr"/>
@@ -9612,7 +9664,7 @@
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>aucune lecture ne dépasse 30 s  [LotRessource.java GET v1/lot/lots [vide] 30003 ms : apiRequestContext.get: Timeout 30000ms exceeded.]</t>
+          <t>aucune lecture ne dépasse 30 s  [LotRessource.java GET v1/lot/lots [vide] 30008 ms : apiRequestContext.get: Timeout 30000ms exceeded.]</t>
         </is>
       </c>
       <c r="E249" s="5" t="inlineStr">
@@ -9644,7 +9696,7 @@
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>aucune nouvelle erreur au Centre de support  [JAVA Blocage détecté : requête en traitement depuis 26s : POST /prestige/api/v1/vente (POST /prestige/api/v1/vente/ticket/vno)]</t>
+          <t>aucune nouvelle erreur au Centre de support  [JAVA Blocage détecté : requête en traitement depuis 26s : GET /prestige/api/v1/fichea (GET /prestige/api/v1/fichearticle/comparaison/excel)]</t>
         </is>
       </c>
       <c r="E250" s="5" t="inlineStr">
@@ -10240,17 +10292,21 @@
           <t>retours/test-ventes-terminees-colonnes.js</t>
         </is>
       </c>
-      <c r="B278" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B278" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C278" s="5" t="inlineStr">
         <is>
-          <t>14 / 14</t>
-        </is>
-      </c>
-      <c r="D278" s="5" t="inlineStr"/>
+          <t>13 / 14</t>
+        </is>
+      </c>
+      <c r="D278" s="5" t="inlineStr">
+        <is>
+          <t>Colonne « P » : vente sans poste connu → vide, encaissement dans l'infobulle  [{"texte":"RM","qtip":"Saisie : RM&lt;br&gt;Encaissement : RM"}]</t>
+        </is>
+      </c>
       <c r="E278" s="5" t="inlineStr"/>
       <c r="F278" s="5" t="inlineStr"/>
     </row>
@@ -10360,27 +10416,19 @@
           <t>retours/test-whatsapp-web.js</t>
         </is>
       </c>
-      <c r="B284" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C284" s="5" t="inlineStr"/>
-      <c r="D284" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E284" s="5" t="inlineStr">
-        <is>
-          <t>Configuration du poste</t>
-        </is>
-      </c>
-      <c r="F284" s="5" t="inlineStr">
-        <is>
-          <t>Service WhatsApp Web (outils/whatsapp-web) non installé sur le poste.</t>
-        </is>
-      </c>
+      <c r="B284" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C284" s="5" t="inlineStr">
+        <is>
+          <t>16 / 16</t>
+        </is>
+      </c>
+      <c r="D284" s="5" t="inlineStr"/>
+      <c r="E284" s="5" t="inlineStr"/>
+      <c r="F284" s="5" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="5" t="inlineStr">
@@ -10395,7 +10443,7 @@
       </c>
       <c r="C285" s="5" t="inlineStr">
         <is>
-          <t>16 / 25</t>
+          <t>17 / 26</t>
         </is>
       </c>
       <c r="D285" s="5" t="inlineStr">
@@ -10447,7 +10495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13 tests, 11 OK, 2 en échec</t>
+          <t>13 tests, 12 OK, 1 en échec</t>
         </is>
       </c>
     </row>
@@ -10629,31 +10677,19 @@
           <t>securite/test-horloge.js</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>2 / 5</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Précondition : horloge du serveur juste, fuseau attendu (Africa/Abidjan), heure d'Internet joignable  [{"fuseau":"Etc/UTC","reference":null,"anomalies":[]}]</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Configuration du poste</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Serveur en UTC alors que le test attend Africa/Abidjan (même heure) et un accès à l'heure d'Internet.</t>
-        </is>
-      </c>
+          <t>11 / 11</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -10748,12 +10784,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>2 / 3</t>
+          <t>4 / 5</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Parcours sans exception  [page.click: Timeout 30000ms exceeded.</t>
+          <t>« Terminer la vente » : vente en dépôt terminée par admin, aucun refus du serveur  [is_Closed|e2e | réponses 200 | Impression du ticketVoulez-vous imprimer le ticket ?OKOuiNonAnnuler]</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -11183,7 +11219,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Onglet Expérience utilisateur : courbe, par poste, écrans et appels les plus lents  [{"serie":20,"postes":1,"ecrans":["RapportGestions","comparaisonChiffreAffaireManager","statfamilleartcl","analysearticle","analyseFrequentationOffManager","articlevendurecapitulatif","activitiessummary","pointagebl","pilotage","mouvementprixvente","statistiqueuniteventemanager","pososmanager","analy]</t>
+          <t>Onglet Expérience utilisateur : courbe, par poste, écrans et appels les plus lents  [{"serie":24,"postes":1,"ecrans":["RapportGestions","comparaisonChiffreAffaireManager","statfamilleartcl","articlevendurecapitulatif","analysearticle","analyseFrequentationOffManager","mouvementprixvente","activitiessummary","pilotage","statistiqueuniteventemanager","analysetierspayant","gestioncaiss]</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -11459,7 +11495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 tests, 3 OK, 0 en échec</t>
+          <t>3 tests, 2 OK, 1 en échec</t>
         </is>
       </c>
     </row>
@@ -11501,17 +11537,21 @@
           <t>audit/test-audit-analyse.js</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>17 / 17</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
+          <t>16 / 17</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Analyse à l'ouverture en moins de 10 s avec 300 clients en différé et 7200 règlements  [{"ms":11040}]</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
@@ -11588,7 +11628,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14 tests, 14 OK, 0 en échec</t>
+          <t>14 tests, 13 OK, 1 en échec</t>
         </is>
       </c>
     </row>
@@ -11850,17 +11890,21 @@
           <t>audits/test-ecran-modifier-vente-deja-modifiee.js</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Échec</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>6 / 6</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr"/>
+          <t>1 / 3</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Préparation : vente modifiée, copie clôturée  [ {"s":false}]</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr"/>
     </row>
@@ -11875,7 +11919,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>10 / 10</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr"/>
@@ -12042,7 +12090,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8 tests, 4 OK, 4 en échec</t>
+          <t>8 tests, 7 OK, 1 en échec</t>
         </is>
       </c>
     </row>
@@ -12084,27 +12132,19 @@
           <t>campagnes/test-campagne-piece-jointe.js</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>arrêt du test (code 1) sans contrôle en échec</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Configuration du poste</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Service WhatsApp Web non installé sur le poste.</t>
-        </is>
-      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>21 / 21</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -12132,31 +12172,19 @@
           <t>campagnes/test-campagnes-destinataires-demande.js</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>3 / 4</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Parcours sans exception  [page.waitForFunction: Timeout 60000ms exceeded.</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+          <t>5 / 5</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -12231,7 +12259,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>8 / 15</t>
+          <t>21 / 27</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -12256,31 +12284,19 @@
           <t>campagnes/test-whatsapp-discussions.js</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>3 / 4</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Parcours sans exception  [locator.click: Timeout 30000ms exceeded.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>À examiner</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
-        </is>
-      </c>
+          <t>15 / 15</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Cahier de recette complet des 422 tests d'écran : scénario, contrôles et résultat obtenu par l'exécution automatique, colonnes du testeur et concordance ; rapport à 366 / 422 après relance des tests touchés par l'arrêt des serveurs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
+++ b/docs/recette/RAPPORT_TESTS_ECRAN_2026-10-30.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -557,7 +557,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>422 tests : 352 OK, 70 en échec</t>
+          <t>422 tests : 366 OK, 56 en échec</t>
         </is>
       </c>
     </row>
@@ -625,10 +625,10 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -641,10 +641,10 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -865,10 +865,10 @@
         <v>12</v>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -977,10 +977,10 @@
         <v>6</v>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1041,10 +1041,10 @@
         <v>282</v>
       </c>
       <c r="C33" t="n">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="D33" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34">
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41">
@@ -1168,10 +1168,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Données d'essai</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Test manuel</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B45" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2149,7 +2159,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12 tests, 9 OK, 3 en échec</t>
+          <t>12 tests, 10 OK, 2 en échec</t>
         </is>
       </c>
     </row>
@@ -2211,21 +2221,17 @@
           <t>journal/test-export-journal.js</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>3 / 6</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>le bouton declenche bien un telechargement  [aucun]</t>
-        </is>
-      </c>
+          <t>10 / 10</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
@@ -2310,8 +2316,16 @@
           <t>Vente dépôt : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé  [{"champ":"htt","fenetre":false,"texte":false} appels : ]</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>À examiner</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Partie « vente dépôt » en échec deux fois de suite l'après-midi (champ partiellement saisi) ; passait le matin.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -3565,7 +3579,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6 tests, 4 OK, 2 en échec</t>
+          <t>6 tests, 6 OK, 0 en échec</t>
         </is>
       </c>
     </row>
@@ -3607,21 +3621,17 @@
           <t>productivite/test-activite-equipes-analyses.js</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>10 / 11</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Parcours sans exception  [page.fill: Timeout 30000ms exceeded.</t>
-        </is>
-      </c>
+          <t>11 / 11</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
@@ -3631,21 +3641,17 @@
           <t>productivite/test-activite-equipes-donnees.js</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0 / 1</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Parcours sans exception  [locator.click: Timeout 30000ms exceeded.</t>
-        </is>
-      </c>
+          <t>11 / 11</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
@@ -4314,7 +4320,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>282 tests, 233 OK, 49 en échec</t>
+          <t>282 tests, 242 OK, 40 en échec</t>
         </is>
       </c>
     </row>
@@ -4852,21 +4858,17 @@
           <t>retours/test-commande-en-cours-0825.js</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>1 / 2</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Parcours sans exception  [locator.click: Timeout 30000ms exceeded.</t>
-        </is>
-      </c>
+          <t>5 / 5</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="5" t="inlineStr"/>
     </row>
@@ -4944,21 +4946,17 @@
           <t>retours/test-connexion-badge-lecture.js</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>8 / 10</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>QWERTY et verrouillage majuscules (« PRESTIGE°BQDGE*1*WWL°2… ») : connexion par le bouton badge  [http://localhost:8080/prestige/security/index.html]</t>
-        </is>
-      </c>
+          <t>11 / 11</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr"/>
       <c r="F31" s="5" t="inlineStr"/>
     </row>
@@ -5357,18 +5355,22 @@
           <t>Échec</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>12 / 12</t>
-        </is>
-      </c>
+      <c r="C49" s="5" t="inlineStr"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
           <t>arrêt du test (code 1) sans contrôle en échec</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Données d'essai</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -5656,21 +5658,17 @@
           <t>retours/test-etiquettes-gs1.js</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>1 / 3</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
-        </is>
-      </c>
+          <t>17 / 17</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr"/>
       <c r="E64" s="5" t="inlineStr"/>
       <c r="F64" s="5" t="inlineStr"/>
     </row>
@@ -5680,21 +5678,17 @@
           <t>retours/test-etiquettes-personnalisation.js</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>1 / 2</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
-        </is>
-      </c>
+          <t>50 / 50</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr"/>
       <c r="E65" s="5" t="inlineStr"/>
       <c r="F65" s="5" t="inlineStr"/>
     </row>
@@ -5953,18 +5947,22 @@
           <t>Échec</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>11 / 11</t>
-        </is>
-      </c>
+      <c r="C77" s="5" t="inlineStr"/>
       <c r="D77" s="5" t="inlineStr">
         <is>
           <t>arrêt du test (code 1) sans contrôle en échec</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr"/>
-      <c r="F77" s="5" t="inlineStr"/>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Données d'essai</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -6060,21 +6058,17 @@
           <t>retours/test-gs1-bascule.js</t>
         </is>
       </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>2 / 4</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
-        </is>
-      </c>
+          <t>25 / 25</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr"/>
       <c r="E82" s="5" t="inlineStr"/>
       <c r="F82" s="5" t="inlineStr"/>
     </row>
@@ -6084,21 +6078,17 @@
           <t>retours/test-gs1-controle-lot.js</t>
         </is>
       </c>
-      <c r="B83" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>2 / 4</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
-        </is>
-      </c>
+          <t>25 / 25</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr"/>
       <c r="E83" s="5" t="inlineStr"/>
       <c r="F83" s="5" t="inlineStr"/>
     </row>
@@ -6472,21 +6462,17 @@
           <t>retours/test-journal-complet.js</t>
         </is>
       </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>1 / 3</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>Déroulement du test  [Error: Command failed: mariadb --defaults-extra-file=C:/Users/AIRMAN/AppData/Local/Temp/claude/D--projet-p3-prestige/4660ea01-cd8f-49ab-bd78-f6382d44836c/scratchpad/e2e-1776.cnf --default-character-set=utf8mb4 laborex_v1_db -sN</t>
-        </is>
-      </c>
+          <t>18 / 18</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr"/>
       <c r="E101" s="5" t="inlineStr"/>
       <c r="F101" s="5" t="inlineStr"/>
     </row>
@@ -6800,21 +6786,17 @@
           <t>retours/test-lot-l.js</t>
         </is>
       </c>
-      <c r="B116" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>30 / 31</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr">
-        <is>
-          <t>jeu d essai pose sur une fenetre vierge (2023-10-01 .. 2023-11-30)  [mouvements preexistants=10]</t>
-        </is>
-      </c>
+          <t>31 / 31</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr"/>
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="5" t="inlineStr"/>
     </row>
@@ -7827,8 +7809,16 @@
           <t>arrêt du test (code 1) sans contrôle en échec</t>
         </is>
       </c>
-      <c r="E163" s="5" t="inlineStr"/>
-      <c r="F163" s="5" t="inlineStr"/>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>Données d'essai</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
@@ -10292,21 +10282,17 @@
           <t>retours/test-ventes-terminees-colonnes.js</t>
         </is>
       </c>
-      <c r="B278" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B278" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C278" s="5" t="inlineStr">
         <is>
-          <t>13 / 14</t>
-        </is>
-      </c>
-      <c r="D278" s="5" t="inlineStr">
-        <is>
-          <t>Colonne « P » : vente sans poste connu → vide, encaissement dans l'infobulle  [{"texte":"RM","qtip":"Saisie : RM&lt;br&gt;Encaissement : RM"}]</t>
-        </is>
-      </c>
+          <t>14 / 14</t>
+        </is>
+      </c>
+      <c r="D278" s="5" t="inlineStr"/>
       <c r="E278" s="5" t="inlineStr"/>
       <c r="F278" s="5" t="inlineStr"/>
     </row>
@@ -11495,7 +11481,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3 tests, 2 OK, 1 en échec</t>
+          <t>3 tests, 3 OK, 0 en échec</t>
         </is>
       </c>
     </row>
@@ -11537,21 +11523,17 @@
           <t>audit/test-audit-analyse.js</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>16 / 17</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Analyse à l'ouverture en moins de 10 s avec 300 clients en différé et 7200 règlements  [{"ms":11040}]</t>
-        </is>
-      </c>
+          <t>17 / 17</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
@@ -11628,7 +11610,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14 tests, 13 OK, 1 en échec</t>
+          <t>14 tests, 14 OK, 0 en échec</t>
         </is>
       </c>
     </row>
@@ -11890,21 +11872,17 @@
           <t>audits/test-ecran-modifier-vente-deja-modifiee.js</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Échec</t>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>1 / 3</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Préparation : vente modifiée, copie clôturée  [ {"s":false}]</t>
-        </is>
-      </c>
+          <t>6 / 6</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
       <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr"/>
     </row>

</xml_diff>